<commit_message>
20 May 2026 - Sync
</commit_message>
<xml_diff>
--- a/items.xlsx
+++ b/items.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ichorsystems-my.sharepoint.com/personal/kmageshkumar_ichorsystems_com/Documents/Scripts/WD Refresher Webpage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{E51FFB5F-9201-4B57-A80B-6D7385D27474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E52631B3-177E-46D2-88BB-B80B2A4F46AF}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{E51FFB5F-9201-4B57-A80B-6D7385D27474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17275656-B763-49F2-8643-7538E23B5B7F}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3C9C76A4-9DD7-4B1A-99C7-4386631A046D}"/>
   </bookViews>
@@ -36,63 +36,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
-  <si>
-    <t>407797N33-EY3-GPB</t>
-  </si>
-  <si>
-    <t>511354-DG-GPA</t>
-  </si>
-  <si>
-    <t>511354-DG-GPB</t>
-  </si>
-  <si>
-    <t>511354-DG-GPC</t>
-  </si>
-  <si>
-    <t>511636-DG-GPA</t>
-  </si>
-  <si>
-    <t>511636-DG-GPB</t>
-  </si>
-  <si>
-    <t>511636-DG-GPC</t>
-  </si>
-  <si>
-    <t>0010-28809</t>
-  </si>
-  <si>
-    <t>0011-02879</t>
-  </si>
-  <si>
-    <t>0011-02880</t>
-  </si>
-  <si>
-    <t>0011-02919</t>
-  </si>
-  <si>
-    <t>0011-06401</t>
-  </si>
-  <si>
-    <t>0246-59922</t>
-  </si>
-  <si>
-    <t>0246-81628</t>
-  </si>
-  <si>
-    <t>0248-04726</t>
-  </si>
-  <si>
-    <t>C02160-ES1-GPA</t>
-  </si>
-  <si>
-    <t>C02160-ES1-GPB</t>
-  </si>
-  <si>
-    <t>C02160-ES1-GPC</t>
-  </si>
-  <si>
-    <t>C02160-ES1-GPD</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>510383-DG-GPB</t>
+  </si>
+  <si>
+    <t>510383-DG-GPC</t>
+  </si>
+  <si>
+    <t>511415-DG-GPA</t>
+  </si>
+  <si>
+    <t>511415-DG-GPB</t>
+  </si>
+  <si>
+    <t>511415-DG-GPC</t>
+  </si>
+  <si>
+    <t>511613-DG-GPC</t>
   </si>
 </sst>
 </file>
@@ -145,10 +106,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -468,102 +425,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32815408-94D6-4190-BD0E-79B70BB6BB23}">
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added feature to delete items under kitting and decon
</commit_message>
<xml_diff>
--- a/items.xlsx
+++ b/items.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ichorsystems-my.sharepoint.com/personal/kmageshkumar_ichorsystems_com/Documents/Scripts/WD Refresher Webpage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{E51FFB5F-9201-4B57-A80B-6D7385D27474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17275656-B763-49F2-8643-7538E23B5B7F}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{E51FFB5F-9201-4B57-A80B-6D7385D27474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECE1C120-E46A-479B-A0B6-DA2C4D37B6A4}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3C9C76A4-9DD7-4B1A-99C7-4386631A046D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3C9C76A4-9DD7-4B1A-99C7-4386631A046D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,22 +38,22 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
-    <t>510383-DG-GPB</t>
-  </si>
-  <si>
-    <t>510383-DG-GPC</t>
-  </si>
-  <si>
-    <t>511415-DG-GPA</t>
-  </si>
-  <si>
-    <t>511415-DG-GPB</t>
-  </si>
-  <si>
-    <t>511415-DG-GPC</t>
-  </si>
-  <si>
-    <t>511613-DG-GPC</t>
+    <t>416742R02-DG-GPA</t>
+  </si>
+  <si>
+    <t>403040R03-DF-GPA</t>
+  </si>
+  <si>
+    <t>420954R10-DG-GPB</t>
+  </si>
+  <si>
+    <t>571-065780-S3836C</t>
+  </si>
+  <si>
+    <t>4022-717-62881-SPARE</t>
+  </si>
+  <si>
+    <t>4022-7182</t>
   </si>
 </sst>
 </file>
@@ -106,6 +106,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -430,17 +434,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -450,7 +454,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added feature to detect >8 versions
</commit_message>
<xml_diff>
--- a/items.xlsx
+++ b/items.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ichorsystems-my.sharepoint.com/personal/kmageshkumar_ichorsystems_com/Documents/Scripts/WD Refresher Webpage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{E51FFB5F-9201-4B57-A80B-6D7385D27474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECE1C120-E46A-479B-A0B6-DA2C4D37B6A4}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{E51FFB5F-9201-4B57-A80B-6D7385D27474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5403A098-9CDF-484B-9426-6E67516FF4EE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3C9C76A4-9DD7-4B1A-99C7-4386631A046D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3C9C76A4-9DD7-4B1A-99C7-4386631A046D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,24 +36,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
-    <t>416742R02-DG-GPA</t>
-  </si>
-  <si>
-    <t>403040R03-DF-GPA</t>
-  </si>
-  <si>
-    <t>420954R10-DG-GPB</t>
-  </si>
-  <si>
-    <t>571-065780-S3836C</t>
-  </si>
-  <si>
-    <t>4022-717-62881-SPARE</t>
-  </si>
-  <si>
-    <t>4022-7182</t>
+    <t>4022-717-32441</t>
   </si>
 </sst>
 </file>
@@ -106,10 +91,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -429,37 +410,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32815408-94D6-4190-BD0E-79B70BB6BB23}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
         <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>